<commit_message>
Add GitHub Pages deployment CI/CD workflow, Selenium Page Object Model, and live E2E testing framework
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Execution Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary Metrics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Live Test Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Risk Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,8 +46,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
     <fill>
@@ -451,7 +451,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Test Case Name</t>
+          <t>Test Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -466,24 +466,24 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Execution Time</t>
+          <t>Target Live URL</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Error Log</t>
+          <t>Timestamp</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TC_001</t>
+          <t>SEL_001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>User Registration &amp; Auth Login</t>
+          <t>Verify Deployed Live URL (HTTP 200)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -492,24 +492,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.25</v>
+        <v>0.35</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-25 22:39:50</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://saishirumala.github.io/PDD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-08-25 22:44:17</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TC_002</t>
+          <t>SEL_002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AI Meal Visual Recognition &amp; Calorie Parse</t>
+          <t>Landing Page Rendering &amp; Hero Elements</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -518,24 +522,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.8</v>
+        <v>1.42</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-25 22:39:50</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://saishirumala.github.io/PDD</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-08-25 22:44:17</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TC_003</t>
+          <t>SEL_003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Water Tracker Quick Add (+250ml)</t>
+          <t>Auth Page Route Navigation</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -544,24 +552,28 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-25 22:39:50</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://saishirumala.github.io/PDD</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-08-25 22:44:17</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TC_004</t>
+          <t>SEL_004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Profile Daily Calorie Target Update</t>
+          <t>Dashboard Page Route Navigation</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -570,14 +582,18 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.1</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-25 22:39:50</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://saishirumala.github.io/PDD</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-08-25 22:44:17</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -590,49 +606,47 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Live Target Base URL</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>https://saishirumala.github.io/PDD</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Build Number</t>
+          <t>Execution Date</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2026-08-25 22:44:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Execution Date</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-08-25 22:39:50</t>
-        </is>
+          <t>Total Live Selenium Tests</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Total Test Cases</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -642,30 +656,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
           <t>Pass Rate</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>

</xml_diff>